<commit_message>
fix(users): prevent duplicate Excel import values
</commit_message>
<xml_diff>
--- a/public/templates/wms-kullanici-aktarim-sablonu.xlsx
+++ b/public/templates/wms-kullanici-aktarim-sablonu.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanıcılar" sheetId="1" r:id="Re0f3bf1504684263"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Açıklamalar" sheetId="2" r:id="Rf418703dcc6d49cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Örnek" sheetId="3" r:id="R28233d0d95b542fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanıcılar" sheetId="1" r:id="R1858a9cd1d3d4255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Açıklamalar" sheetId="2" r:id="R017155a8afc84158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Örnek" sheetId="3" r:id="Rc3807789aacd4a35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -456,6 +456,30 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="2">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
@@ -1014,11 +1038,27 @@
       <x:c r="I30" s="27"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="G2:G1000">
+  <x:conditionalFormatting sqref="A2:A501">
+    <x:cfRule type="expression" dxfId="0" priority="1">
+      <x:formula>AND(A2&lt;&gt;"",COUNTIF($A$2:$A$501,A2)&gt;1)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="B2:B501">
+    <x:cfRule type="expression" dxfId="1" priority="2">
+      <x:formula>AND(B2&lt;&gt;"",COUNTIF($B$2:$B$501,B2)&gt;1)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="4">
+    <x:dataValidation type="custom" errorStyle="stop" showInputMessage="1" showErrorMessage="1" errorTitle="Mükerrer kullanıcı adı" error="Bu kullanıcı adı dosyada zaten kullanılmış. Benzersiz bir kullanıcı adı girin." promptTitle="Benzersiz kullanıcı adı" prompt="Bu sütunda aynı kullanıcı adı yalnızca bir kez kullanılabilir." sqref="A2:A501">
+      <x:formula1>OR(A2="",COUNTIF($A$2:$A$501,A2)=1)</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="custom" errorStyle="stop" showInputMessage="1" showErrorMessage="1" errorTitle="Mükerrer e-posta" error="Bu e-posta adresi dosyada zaten kullanılmış. Benzersiz bir e-posta girin." promptTitle="Benzersiz e-posta" prompt="Bu sütunda aynı e-posta adresi yalnızca bir kez kullanılabilir." sqref="B2:B501">
+      <x:formula1>OR(B2="",COUNTIF($B$2:$B$501,B2)=1)</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G2:G501">
       <x:formula1>"User,Manager,Admin"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="H2:H1000">
+    <x:dataValidation type="list" sqref="H2:H501">
       <x:formula1>"true,false"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -1050,7 +1090,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="45" t="str">
-        <x:v>ÖNEMLİ: Bu aktarım yalnızca yeni kullanıcı kaydı oluşturur. Mevcut kullanıcıları güncellemez, pasife almaz veya silmez. Mevcut kullanıcı adı/e-posta ile dosya içindeki mükerrer satırlar atlanır.</x:v>
+        <x:v>ÖNEMLİ: Bu aktarım yalnızca yeni kullanıcı kaydı oluşturur. Mevcut kullanıcıları güncellemez, pasife almaz veya silmez. Excel aynı kullanıcı adı/e-postanın tekrarını engeller; kopyala-yapıştır ile oluşan tekrarları kırmızı işaretler. API son kontrolde mükerrer satırları atlar.</x:v>
       </x:c>
       <x:c r="B3" s="46"/>
       <x:c r="C3" s="46"/>
@@ -1100,10 +1140,10 @@
         <x:v>ayse.yilmaz</x:v>
       </x:c>
       <x:c r="E7" s="61" t="str">
-        <x:v>Harf, rakam, nokta, tire ve alt çizgi</x:v>
+        <x:v>Dosya içinde benzersiz; harf, rakam, nokta, tire ve alt çizgi</x:v>
       </x:c>
       <x:c r="F7" s="61" t="str">
-        <x:v>Mevcutsa satır atlanır</x:v>
+        <x:v>Sistemde mevcutsa satır atlanır</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="35" customHeight="1">
@@ -1120,10 +1160,10 @@
         <x:v>ayse.yilmaz@firma.com</x:v>
       </x:c>
       <x:c r="E8" s="62" t="str">
-        <x:v>En fazla 200 karakter</x:v>
+        <x:v>Dosya içinde benzersiz; en fazla 200 karakter</x:v>
       </x:c>
       <x:c r="F8" s="62" t="str">
-        <x:v>Mevcutsa satır atlanır</x:v>
+        <x:v>Sistemde mevcutsa satır atlanır</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="35" customHeight="1">

</xml_diff>

<commit_message>
docs(users): align import template password policy
</commit_message>
<xml_diff>
--- a/public/templates/wms-kullanici-aktarim-sablonu.xlsx
+++ b/public/templates/wms-kullanici-aktarim-sablonu.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanıcılar" sheetId="1" r:id="R1858a9cd1d3d4255"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Açıklamalar" sheetId="2" r:id="R017155a8afc84158"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Örnek" sheetId="3" r:id="Rc3807789aacd4a35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kullanıcılar" sheetId="1" r:id="Ra6df41fa0bed4cf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Açıklamalar" sheetId="2" r:id="R2fd2e5fed96c4e94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Örnek" sheetId="3" r:id="Ra1a82c1453e44ef0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1174,13 +1174,13 @@
         <x:v>Evet</x:v>
       </x:c>
       <x:c r="C9" s="62" t="str">
-        <x:v>15-128 karakter</x:v>
+        <x:v>Genel Ayarlar min.-15</x:v>
       </x:c>
       <x:c r="D9" s="62" t="str">
-        <x:v>Gecici!Sifre2026</x:v>
+        <x:v>Gecici!2026</x:v>
       </x:c>
       <x:c r="E9" s="62" t="str">
-        <x:v>Uygulamanın şifre politikasına uymalı</x:v>
+        <x:v>Yükleme anındaki merkezi şifre politikasına uymalı</x:v>
       </x:c>
       <x:c r="F9" s="62" t="str">
         <x:v>Sonuçlarda ve loglarda gösterilmez</x:v>
@@ -1380,7 +1380,7 @@
         <x:v>ayse.yilmaz@firma.com</x:v>
       </x:c>
       <x:c r="C2" s="86" t="str">
-        <x:v>Gecici!Sifre2026</x:v>
+        <x:v>Gecici!2026</x:v>
       </x:c>
       <x:c r="D2" s="86" t="str">
         <x:v>Ayşe</x:v>

</xml_diff>